<commit_message>
Add address column to clients Excel import template
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/static/templates/clients_template.xlsx
+++ b/static/templates/clients_template.xlsx
@@ -28,30 +28,35 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>رقم الهاتف</t>
+          <t>العنوان</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>البريد الإلكتروني</t>
+          <t>رقم الهاتف</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>اسم المسؤول</t>
+          <t>البريد الإلكتروني</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>نوع المتعاقد</t>
+          <t>اسم المسؤول</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>نوع المتعاقد</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>رقم هوية المتعاقد</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>رقم السجل التجاري</t>
         </is>

</xml_diff>